<commit_message>
Expand marketing dashboard KPI analysis
</commit_message>
<xml_diff>
--- a/public/medi-insight-google-sheets-template.xlsx
+++ b/public/medi-insight-google-sheets-template.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="입력안내" sheetId="1" r:id="rId1"/>
-    <sheet name="상담문의" sheetId="2" r:id="rId2"/>
-    <sheet name="예약" sheetId="3" r:id="rId3"/>
-    <sheet name="내원" sheetId="4" r:id="rId4"/>
-    <sheet name="결제매출" sheetId="5" r:id="rId5"/>
-    <sheet name="광고비" sheetId="6" r:id="rId6"/>
+    <sheet name="추가항목 안내" sheetId="1" r:id="rId1"/>
+    <sheet name="입력안내" sheetId="2" r:id="rId2"/>
+    <sheet name="상담문의" sheetId="3" r:id="rId3"/>
+    <sheet name="예약" sheetId="4" r:id="rId4"/>
+    <sheet name="내원" sheetId="5" r:id="rId5"/>
+    <sheet name="결제매출" sheetId="6" r:id="rId6"/>
+    <sheet name="광고비" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -17,108 +18,359 @@
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>메디인사이트 Google Sheets 입력 템플릿</t>
+          <t>테이블</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>영문 열 이름</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>한글 항목</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>입력 예시</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>활용</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>구분</t>
+          <t>상담문의</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>내용</t>
+          <t>chart_number</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>차트번호/공통 연결키</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>C-8F31A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>상담-예약-내원-결제 직접 연결 및 퍼널 대사</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1행</t>
+          <t>상담문의</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>영문 시스템 컬럼입니다. 앱 동기화가 이 값을 기준으로 읽으므로 수정하지 마세요.</t>
+          <t>consult_result</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>상담결과</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>예약확정 / 미예약</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>예약확정, 미예약 운영 지표</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2행</t>
+          <t>내원</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>한글 항목명입니다. 입력자가 이해하기 위한 안내 행입니다.</t>
+          <t>visit_setting</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>방문형태</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>예약내원 / 비예약내원</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>비예약 내원 분석</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3행</t>
+          <t>내원</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>각 항목의 설명입니다. 실제 데이터로 저장되지 않습니다.</t>
+          <t>care_setting</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>진료구분</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>외래 / 입원</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>외래·입원 전환 분석</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4행</t>
+          <t>광고비</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>예시 값입니다. 실제 데이터로 저장되지 않습니다.</t>
+          <t>cost_type</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>비용구분</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>online / crm / fixed</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>통합 광고비 = 온라인 + CRM + 고정</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5행부터</t>
+          <t>광고비</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>실제 운영 데이터를 입력하세요. 구글 시트 동기화 시 5행부터만 반영됩니다.</t>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>진료분야</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>교통사고</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>진료분야별 광고비, CPL, 신환당 비용, ROAS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>탭 이름</t>
+          <t>광고비</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>상담문의, 예약, 내원, 결제매출, 광고비 탭 이름은 변경하지 마세요.</t>
+          <t>sent_count</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CRM 발송수</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CRM 발송당 비용과 발송 대비 예약률</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>개인정보</t>
+          <t>광고비</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>이름, 전화번호 등 개인정보 대신 환자 가명키를 사용하세요.</t>
+          <t>crm_inquiries</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CRM 문의수</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CRM 문의율과 문의당 비용</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>광고비</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>crm_reservations</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CRM 예약수</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CRM 예약당 비용</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>광고비</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>crm_paid_customers</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CRM 결제고객수</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CRM 결제고객당 비용</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>광고비</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>fixed_contract_end</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>고정비 계약종료일</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>계약 종료 예정 비용 관리</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>주의</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>연결 규칙</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>lead_id → appointment_id → visit_id → payment_id</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>기간 합계와 세부 합계 자동 대사</t>
         </is>
       </c>
     </row>
@@ -127,6 +379,120 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>메디인사이트 Google Sheets 입력 템플릿</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1행</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>영문 시스템 컬럼입니다. 앱 동기화가 이 값을 기준으로 읽으므로 수정하지 마세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2행</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>한글 항목명입니다. 입력자가 이해하기 위한 안내 행입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3행</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>각 항목의 설명입니다. 실제 데이터로 저장되지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4행</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>예시 값입니다. 실제 데이터로 저장되지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5행부터</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>실제 운영 데이터를 입력하세요. 구글 시트 동기화 시 5행부터만 반영됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>탭 이름</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>상담문의, 예약, 내원, 결제매출, 광고비 탭 이름은 변경하지 마세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>개인정보</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>이름, 전화번호 등 개인정보 대신 환자 가명키를 사용하세요.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -346,191 +712,6 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>예약완료</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>appointment_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>lead_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>patient_key</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>booked_at</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>scheduled_at</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>department</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>cancel_reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>예약 ID</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>문의 ID</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>환자 가명키</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>예약 확정 일시</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>방문 예정 일시</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>예약 진료과목</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>예약 상태</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>취소 사유</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>필수. 예약 건을 구분하는 고유값입니다.</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>선택. 상담문의 시트의 문의 ID와 연결합니다.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>선택. 환자 단위 중복 분석용 키입니다.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>필수. 예약이 확정된 날짜와 시간입니다.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>필수. 실제 내원 예정 날짜와 시간입니다.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>필수. 예약된 진료과목입니다.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>필수. 예약확정, 변경, 취소, 노쇼, 내원완료 중 입력합니다.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>선택. 취소 또는 노쇼 사유를 입력합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>A-20260720-001</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>L-20260720-001</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>P-8F31A</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-07-20 10:02</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-21 15:30</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>수술후재활</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>예약확정</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>일정 변경</t>
         </is>
       </c>
     </row>
@@ -554,12 +735,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>visit_id</t>
+          <t>appointment_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>appointment_id</t>
+          <t>lead_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -569,12 +750,12 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>visited_at</t>
+          <t>booked_at</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>visit_type</t>
+          <t>scheduled_at</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -584,24 +765,24 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>treatment_type</t>
+          <t>status</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>visit_source</t>
+          <t>cancel_reason</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>내원 ID</t>
+          <t>예약 ID</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>예약 ID</t>
+          <t>문의 ID</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -611,81 +792,81 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>내원 일시</t>
+          <t>예약 확정 일시</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>내원 구분</t>
+          <t>방문 예정 일시</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>내원 진료과목</t>
+          <t>예약 진료과목</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>치료 유형</t>
+          <t>예약 상태</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>내원 경로</t>
+          <t>취소 사유</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>필수. 내원 건을 구분하는 고유값입니다.</t>
+          <t>필수. 예약 건을 구분하는 고유값입니다.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>선택. 예약 후 내원인 경우 예약 ID를 입력합니다.</t>
+          <t>선택. 상담문의 시트의 문의 ID와 연결합니다.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>필수. 신환/재진과 재내원 분석용 키입니다.</t>
+          <t>선택. 환자 단위 중복 분석용 키입니다.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>필수. 실제 방문 완료 날짜와 시간입니다.</t>
+          <t>필수. 예약이 확정된 날짜와 시간입니다.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>필수. 신환 또는 재진을 입력합니다.</t>
+          <t>필수. 실제 내원 예정 날짜와 시간입니다.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>필수. 실제 내원한 진료과목입니다.</t>
+          <t>필수. 예약된 진료과목입니다.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>선택. 내부 치료 또는 프로그램명을 입력합니다.</t>
+          <t>필수. 예약확정, 변경, 취소, 노쇼, 내원완료 중 입력합니다.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>필수. 실제 내원 기준 유입 경로입니다.</t>
+          <t>선택. 취소 또는 노쇼 사유를 입력합니다.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>V-20260721-001</t>
+          <t>A-20260720-001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A-20260720-001</t>
+          <t>L-20260720-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -695,27 +876,27 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-21 15:28</t>
+          <t>2026-07-20 10:02</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>신환</t>
+          <t>2026-07-21 15:30</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>교통사고</t>
+          <t>수술후재활</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>도수치료</t>
+          <t>예약확정</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>카페(청라맘스)</t>
+          <t>일정 변경</t>
         </is>
       </c>
     </row>
@@ -739,12 +920,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>payment_id</t>
+          <t>visit_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>visit_id</t>
+          <t>appointment_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -754,39 +935,39 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>paid_at</t>
+          <t>visited_at</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>gross_amount</t>
+          <t>visit_type</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>refund_amount</t>
+          <t>department</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>net_amount</t>
+          <t>treatment_type</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>department</t>
+          <t>visit_source</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>결제 ID</t>
+          <t>내원 ID</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>내원 ID</t>
+          <t>예약 ID</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -796,81 +977,81 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>결제 일시</t>
+          <t>내원 일시</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>총 결제금액</t>
+          <t>내원 구분</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>환불 금액</t>
+          <t>내원 진료과목</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>순매출</t>
+          <t>치료 유형</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>매출 진료과목</t>
+          <t>내원 경로</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>필수. 결제 건을 구분하는 고유값입니다.</t>
+          <t>필수. 내원 건을 구분하는 고유값입니다.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>선택. 내원 시트의 내원 ID와 연결합니다.</t>
+          <t>선택. 예약 후 내원인 경우 예약 ID를 입력합니다.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>선택. 환자 단위 매출 분석용 키입니다.</t>
+          <t>필수. 신환/재진과 재내원 분석용 키입니다.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>필수. 결제가 완료된 날짜와 시간입니다.</t>
+          <t>필수. 실제 방문 완료 날짜와 시간입니다.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>필수. 환불 전 결제 금액입니다. 숫자만 입력합니다.</t>
+          <t>필수. 신환 또는 재진을 입력합니다.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>필수. 환불 또는 취소 금액입니다. 없으면 0을 입력합니다.</t>
+          <t>필수. 실제 내원한 진료과목입니다.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>필수. 총 결제금액에서 환불 금액을 뺀 금액입니다.</t>
+          <t>선택. 내부 치료 또는 프로그램명을 입력합니다.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>선택. 진료과목별 매출 기여 분석에 사용합니다.</t>
+          <t>필수. 실제 내원 기준 유입 경로입니다.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PAY-20260721-001</t>
+          <t>V-20260721-001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>V-20260721-001</t>
+          <t>A-20260720-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -880,21 +1061,27 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-21 16:10</t>
-        </is>
-      </c>
-      <c r="E4">
-        <v>350000</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>350000</v>
+          <t>2026-07-21 15:28</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>신환</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>교통사고</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>도수치료</t>
+        </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>다이어트</t>
+          <t>카페(청라맘스)</t>
         </is>
       </c>
     </row>
@@ -913,6 +1100,185 @@
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>payment_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>patient_key</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>paid_at</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>gross_amount</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>refund_amount</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>net_amount</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>결제 ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>내원 ID</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>환자 가명키</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>결제 일시</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>총 결제금액</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>환불 금액</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>순매출</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>매출 진료과목</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>필수. 결제 건을 구분하는 고유값입니다.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>선택. 내원 시트의 내원 ID와 연결합니다.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>선택. 환자 단위 매출 분석용 키입니다.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>필수. 결제가 완료된 날짜와 시간입니다.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>필수. 환불 전 결제 금액입니다. 숫자만 입력합니다.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>필수. 환불 또는 취소 금액입니다. 없으면 0을 입력합니다.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>필수. 총 결제금액에서 환불 금액을 뺀 금액입니다.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>선택. 진료과목별 매출 기여 분석에 사용합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PAY-20260721-001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>V-20260721-001</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P-8F31A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-07-21 16:10</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>350000</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>350000</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>다이어트</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>